<commit_message>
Commit 6: Perguntas de Negógios criadas
</commit_message>
<xml_diff>
--- a/Data/1 - Raw/Contratos/Contratos.xlsx
+++ b/Data/1 - Raw/Contratos/Contratos.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F70BB27A-F948-47B4-864C-B66C16140FE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -9516,7 +9516,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -9533,7 +9533,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>

</xml_diff>